<commit_message>
List Ladder: percentile-based tiers per position (Elite top 10%, A-Grade top 30%, B-Grade top 50%)
- Replaced fixed rating thresholds with per-position percentile distribution
- Rating pills use Player Ratings Matrix color system (rating_colour_for_value)
- Tier badges: Elite (dark green), A-Grade (light green), B-Grade (gold), untiered (white)
- Players with 0 matches show NA with grey pill
- Percentile calculation excludes 0-match players for better color distribution
- Updated compute_list_ladder.py with matching percentile logic
- Updated data files with latest 2026 season data
</commit_message>
<xml_diff>
--- a/afl_ladders_2011_2025.xlsx
+++ b/afl_ladders_2011_2025.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N281"/>
+  <dimension ref="A1:N288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14496,17 +14496,17 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Sydney Swans</t>
+          <t>Gold Coast Suns</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -14526,22 +14526,22 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>384</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>201</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>191.30%</t>
+          <t>191.04%</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
@@ -14551,7 +14551,7 @@
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Won 3</t>
         </is>
       </c>
       <c r="N271" t="n">
@@ -14566,17 +14566,17 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Gold Coast Suns</t>
+          <t>Western Bulldogs</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -14596,22 +14596,22 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>339</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>247</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>181.16%</t>
+          <t>137.25%</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
@@ -14621,7 +14621,7 @@
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Won 3</t>
         </is>
       </c>
       <c r="N272" t="n">
@@ -14636,52 +14636,52 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>GWS Giants</t>
+          <t>Sydney Swans</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E273" t="inlineStr">
+      <c r="F273" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>66.67%</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>318</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>228</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>128.42%</t>
+          <t>139.47%</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
@@ -14691,7 +14691,7 @@
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N273" t="n">
@@ -14706,52 +14706,52 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Collingwood Magpies</t>
+          <t>Hawthorn Hawks</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E274" t="inlineStr">
+      <c r="F274" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>66.67%</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>339</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>287</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>118.18%</t>
+          <t>118.12%</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
@@ -14761,7 +14761,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Won 2</t>
         </is>
       </c>
       <c r="N274" t="n">
@@ -14776,62 +14776,62 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Western Bulldogs</t>
+          <t>Geelong Cats</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E275" t="inlineStr">
+      <c r="F275" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>66.67%</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>247</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>285</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>104.72%</t>
+          <t>86.67%</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+9</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Won 2</t>
         </is>
       </c>
       <c r="N275" t="n">
@@ -14846,7 +14846,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Carlton Blues</t>
+          <t>Fremantle Dockers</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -14881,22 +14881,22 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>218</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>180</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>70.94%</t>
+          <t>121.11%</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
@@ -14916,52 +14916,52 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Brisbane Lions</t>
+          <t>North Melbourne Kangaroos</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr">
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F277" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>207</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>178</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>95.50%</t>
+          <t>116.29%</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
@@ -14986,62 +14986,62 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Richmond Tigers</t>
+          <t>Port Adelaide Power</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr">
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F278" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>200</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>183</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>94.67%</t>
+          <t>109.29%</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N278" t="n">
@@ -15056,62 +15056,62 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>St Kilda Saints</t>
+          <t>Adelaide Crows</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D279" t="inlineStr">
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F279" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>33.33%</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>241</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>241</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>84.62%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Lost 2</t>
         </is>
       </c>
       <c r="N279" t="n">
@@ -15126,57 +15126,57 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Hawthorn Hawks</t>
+          <t>Collingwood Magpies</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr">
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F280" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>157</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>159</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>77.87%</t>
+          <t>98.74%</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
@@ -15196,65 +15196,555 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Geelong Cats</t>
+          <t>St Kilda Saints</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D281" t="inlineStr">
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr">
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>251</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>272</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>92.28%</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>Won 1</t>
+        </is>
+      </c>
+      <c r="N281" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Melbourne Demons</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F281" t="inlineStr">
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G281" t="inlineStr">
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>84.44%</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>Lost 1</t>
+        </is>
+      </c>
+      <c r="N282" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>West Coast Eagles</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>81.33%</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>Won 1</t>
+        </is>
+      </c>
+      <c r="N283" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>GWS Giants</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>249</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>307</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>81.11%</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>Lost 2</t>
+        </is>
+      </c>
+      <c r="N284" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Carlton Blues</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>70.94%</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>+0</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>Won 1</t>
+        </is>
+      </c>
+      <c r="N285" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Brisbane Lions</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="H281" t="inlineStr">
+      <c r="H286" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I281" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="J281" t="inlineStr">
-        <is>
-          <t>125</t>
-        </is>
-      </c>
-      <c r="K281" t="inlineStr">
-        <is>
-          <t>55.20%</t>
-        </is>
-      </c>
-      <c r="L281" t="inlineStr">
-        <is>
-          <t>-2</t>
-        </is>
-      </c>
-      <c r="M281" t="inlineStr">
-        <is>
-          <t>Lost 1</t>
-        </is>
-      </c>
-      <c r="N281" t="n">
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>166</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>77.21%</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>+0</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Lost 2</t>
+        </is>
+      </c>
+      <c r="N286" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Richmond Tigers</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>64.53%</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>+0</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Lost 2</t>
+        </is>
+      </c>
+      <c r="N287" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Essendon Bombers</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>153</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>55.04%</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>+0</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Lost 2</t>
+        </is>
+      </c>
+      <c r="N288" t="n">
         <v>2026</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stale ladder data, Traits API season-aware caching & VFL/SANFL fallback
Ladder fixes:
- app.py: load_afl_ladder_positions() prefers scraped data for current season
- data_loader.py: checks data/ subdirectory first for ladder files
- scrape_afl_ladders.py: writes to all 3 output locations
- scheduled_update.py: refresh_master_ladders reads from data/ directory
- Updated master workbook Team_Ladders_All with Round 4 data

Pipeline reliability:
- scheduled_update.py: restarts Streamlit after pipeline run to clear cache

Traits API improvements:
- traits_api.py: parse_traits_response falls back to VFL/SANFL/WAFL
- traits_api.py: removed VFL exclusion from cache lookups
- run_traits_api.py: season-aware cache invalidation
- Coverage improved from 73% to 85% (674/790 players)

Data updates:
- Fresh Round 4 ladder data across all files
- Refreshed Traits API cache with 2026 season data
- Updated computed ratings, team summaries, player stats
</commit_message>
<xml_diff>
--- a/afl_ladders_2011_2025.xlsx
+++ b/afl_ladders_2011_2025.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14496,17 +14496,17 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Gold Coast Suns</t>
+          <t>Western Bulldogs</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -14526,32 +14526,32 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>438</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>312</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>191.04%</t>
+          <t>140.38%</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>Won 3</t>
+          <t>Won 4</t>
         </is>
       </c>
       <c r="N271" t="n">
@@ -14566,32 +14566,32 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Western Bulldogs</t>
+          <t>Sydney Swans</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="E272" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>75.00%</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -14601,27 +14601,27 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>339</t>
+          <t>481</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>263</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>137.25%</t>
+          <t>182.89%</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>Won 3</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N272" t="n">
@@ -14636,19 +14636,19 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Sydney Swans</t>
+          <t>Gold Coast Suns</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="E273" t="inlineStr">
         <is>
           <t>1</t>
@@ -14661,32 +14661,32 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>75.00%</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>318</t>
+          <t>473</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>310</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>139.47%</t>
+          <t>152.58%</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
@@ -14706,19 +14706,19 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Hawthorn Hawks</t>
+          <t>Fremantle Dockers</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="E274" t="inlineStr">
         <is>
           <t>1</t>
@@ -14731,37 +14731,37 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>75.00%</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>339</t>
+          <t>399</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>299</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>118.12%</t>
+          <t>133.44%</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>Won 2</t>
+          <t>Won 3</t>
         </is>
       </c>
       <c r="N274" t="n">
@@ -14776,19 +14776,19 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Geelong Cats</t>
+          <t>North Melbourne Kangaroos</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="E275" t="inlineStr">
         <is>
           <t>1</t>
@@ -14801,32 +14801,32 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>75.00%</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>384</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>333</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>86.67%</t>
+          <t>115.32%</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>+9</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
@@ -14846,24 +14846,24 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Fremantle Dockers</t>
+          <t>Hawthorn Hawks</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="F276" t="inlineStr">
         <is>
           <t>0</t>
@@ -14871,27 +14871,27 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>75.00%</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>431</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>378</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>121.11%</t>
+          <t>114.02%</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Won 3</t>
         </is>
       </c>
       <c r="N276" t="n">
@@ -14916,24 +14916,24 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>North Melbourne Kangaroos</t>
+          <t>Melbourne Demons</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="F277" t="inlineStr">
         <is>
           <t>0</t>
@@ -14941,37 +14941,37 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>75.00%</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>399</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>391</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>116.29%</t>
+          <t>102.05%</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Won 2</t>
         </is>
       </c>
       <c r="N277" t="n">
@@ -14991,17 +14991,17 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -15016,27 +15016,27 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>380</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>323</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>109.29%</t>
+          <t>117.65%</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
@@ -15056,17 +15056,17 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Adelaide Crows</t>
+          <t>Brisbane Lions</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -15081,37 +15081,37 @@
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>398</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>360</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>110.56%</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Lost 2</t>
+          <t>Won 2</t>
         </is>
       </c>
       <c r="N279" t="n">
@@ -15131,17 +15131,17 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -15156,27 +15156,27 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>309</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>332</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>98.74%</t>
+          <t>93.07%</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
@@ -15196,17 +15196,17 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>St Kilda Saints</t>
+          <t>Geelong Cats</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -15221,27 +15221,27 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>338</t>
         </is>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>272</t>
+          <t>377</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>92.28%</t>
+          <t>89.66%</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
@@ -15251,7 +15251,7 @@
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N281" t="n">
@@ -15266,22 +15266,22 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Melbourne Demons</t>
+          <t>West Coast Eagles</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -15296,27 +15296,27 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>310</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>478</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>84.44%</t>
+          <t>64.85%</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
@@ -15336,12 +15336,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>West Coast Eagles</t>
+          <t>Adelaide Crows</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -15351,7 +15351,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -15361,7 +15361,7 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
@@ -15371,17 +15371,17 @@
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>317</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>319</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>81.33%</t>
+          <t>99.37%</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
@@ -15391,7 +15391,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Lost 3</t>
         </is>
       </c>
       <c r="N283" t="n">
@@ -15406,24 +15406,24 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>GWS Giants</t>
+          <t>St Kilda Saints</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D284" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E284" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="F284" t="inlineStr">
         <is>
           <t>0</t>
@@ -15431,7 +15431,7 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
@@ -15441,27 +15441,27 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>331</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>307</t>
+          <t>385</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>81.11%</t>
+          <t>85.97%</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+0</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Lost 2</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N284" t="n">
@@ -15481,7 +15481,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -15491,7 +15491,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -15501,7 +15501,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
@@ -15511,27 +15511,27 @@
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>307</t>
         </is>
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>399</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>70.94%</t>
+          <t>76.94%</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Lost 2</t>
         </is>
       </c>
       <c r="N285" t="n">
@@ -15546,62 +15546,62 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Brisbane Lions</t>
+          <t>GWS Giants</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F286" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>166</t>
+          <t>303</t>
         </is>
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>394</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>77.21%</t>
+          <t>76.90%</t>
         </is>
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>Lost 2</t>
+          <t>Lost 3</t>
         </is>
       </c>
       <c r="N286" t="n">
@@ -15616,12 +15616,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Richmond Tigers</t>
+          <t>Essendon Bombers</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -15631,7 +15631,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -15651,17 +15651,17 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>287</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>458</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>64.53%</t>
+          <t>62.66%</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
@@ -15671,7 +15671,7 @@
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Lost 2</t>
+          <t>Lost 4</t>
         </is>
       </c>
       <c r="N287" t="n">
@@ -15686,12 +15686,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Essendon Bombers</t>
+          <t>Richmond Tigers</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -15701,7 +15701,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -15721,17 +15721,17 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>222</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>396</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>55.04%</t>
+          <t>56.06%</t>
         </is>
       </c>
       <c r="L288" t="inlineStr">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Lost 2</t>
+          <t>Lost 4</t>
         </is>
       </c>
       <c r="N288" t="n">

</xml_diff>